<commit_message>
Sow: remove all website integration (Michael: no site). No default link, no site platform/card/caption, cron no longer marks site, public read policy dropped
</commit_message>
<xml_diff>
--- a/public/template/sow-content-bank-template.xlsx
+++ b/public/template/sow-content-bank-template.xlsx
@@ -545,7 +545,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>facebook, whatsapp, x, youtube, site</t>
+          <t>facebook, whatsapp, x, youtube</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>facebook, whatsapp, site</t>
+          <t>facebook, whatsapp</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Platforms: any of facebook, groups, fb page, whatsapp, channel, x, youtube, site, separated by commas. Empty = everywhere.</t>
+          <t>Platforms: any of facebook, groups, fb page, whatsapp, channel, x, youtube, separated by commas. Empty = everywhere.</t>
         </is>
       </c>
     </row>

</xml_diff>